<commit_message>
added few papers for review & added monthly clearance doc
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\rag-dissertation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2E0BE00B-B0B8-408D-815E-6B3574DDA766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B0DC0FB-7196-4B7A-AE9E-2C477F2756E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F211E78F-65A6-4528-B59A-5C2BEDBB7ED5}"/>
   </bookViews>
@@ -34,16 +34,64 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>LITERATURE REVIEW</t>
+  </si>
+  <si>
+    <t>Paper</t>
+  </si>
+  <si>
+    <t>Subject</t>
+  </si>
+  <si>
+    <t>Outcome</t>
+  </si>
+  <si>
+    <t>S.no.</t>
+  </si>
+  <si>
+    <t>Re2G: Retrieve, Rerank, Generate</t>
+  </si>
+  <si>
+    <t>Publisher</t>
+  </si>
+  <si>
+    <t>Maximizing RAG efficiency: A comparative analysis of RAG methods</t>
+  </si>
+  <si>
+    <r>
+      <t>Cambridge University Press:  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FF333333"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>30 October 2024</t>
+    </r>
+  </si>
+  <si>
+    <t>EvaRAG: Evaluating Advanced RAG Techniques With Indexing and Distance Metrics</t>
+  </si>
+  <si>
+    <t>IEEE</t>
+  </si>
+  <si>
+    <t>TYPED-RAG: Type-Aware Decomposition of Non-Factoid Questions for Retrieval-Augmented Generation</t>
+  </si>
+  <si>
+    <t>Association for Computational Linguistics</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -58,6 +106,40 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="19"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF212529"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -77,14 +159,27 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -397,15 +492,76 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74087FDA-DCB0-42F6-A046-4BB743948387}">
-  <dimension ref="C6"/>
+  <dimension ref="B6:F12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="88.5546875" customWidth="1"/>
+    <col min="4" max="4" width="55.77734375" customWidth="1"/>
+    <col min="5" max="5" width="37.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="6" spans="3:3" ht="31.2" x14ac:dyDescent="0.6">
+    <row r="6" spans="2:6" ht="31.2" x14ac:dyDescent="0.6">
       <c r="C6" s="1" t="s">
         <v>0</v>
       </c>
     </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" t="s">
+        <v>2</v>
+      </c>
+      <c r="F8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B9" s="3">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="48" x14ac:dyDescent="0.3">
+      <c r="C10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="15" x14ac:dyDescent="0.35">
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="15" x14ac:dyDescent="0.35">
+      <c r="C12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C9" r:id="rId1" display="https://aclanthology.org/2022.naacl-main.194.pdf" xr:uid="{68E5C6A5-EDD3-4584-9F9D-6426C53B75D7}"/>
+    <hyperlink ref="C12" r:id="rId2" display="https://aclanthology.org/2022.naacl-main.194.pdf" xr:uid="{69D0E201-038C-4594-A25F-23C3DA1E8BF8}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>